<commit_message>
poprawki mniejsze i szablony nowe
</commit_message>
<xml_diff>
--- a/app/templates/szablon_terminarz.xlsx
+++ b/app/templates/szablon_terminarz.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\radek\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{016AF006-C110-4DDC-8D01-D66708FEF89A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21DE1C5-69AB-4AE5-8C48-A43A7F3380E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-3132" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -435,22 +435,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>436260</xdr:colOff>
+      <xdr:colOff>508000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>46535</xdr:rowOff>
+      <xdr:rowOff>36286</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>391031</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>23268</xdr:rowOff>
+      <xdr:colOff>401569</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>234141</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2087D7CD-454C-DB87-9107-8FE5C0D3C949}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A23E3258-5889-98CC-4637-1BF006105504}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -472,8 +472,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5787710" y="46535"/>
-          <a:ext cx="1990649" cy="1105191"/>
+          <a:off x="5860143" y="36286"/>
+          <a:ext cx="1925569" cy="1086855"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>